<commit_message>
selenium new framework upoaded
</commit_message>
<xml_diff>
--- a/excel/Data.xlsx
+++ b/excel/Data.xlsx
@@ -4,22 +4,19 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="120" windowWidth="20115" windowHeight="7500" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="120" windowWidth="20115" windowHeight="7500" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Credential" sheetId="1" r:id="rId1"/>
     <sheet name="Hotel" sheetId="2" r:id="rId2"/>
-    <sheet name="SelectHotel" sheetId="3" r:id="rId3"/>
+    <sheet name="BookHotel" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="38">
-  <si>
-    <t xml:space="preserve">thiyaguadmin </t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
   <si>
     <t>Admin@123</t>
   </si>
@@ -45,72 +42,33 @@
     <t>Double</t>
   </si>
   <si>
-    <t>Hotel Name</t>
+    <t>2 - Two</t>
+  </si>
+  <si>
+    <t>0 - None</t>
+  </si>
+  <si>
+    <t>3 - Three</t>
+  </si>
+  <si>
+    <t>1 - One</t>
+  </si>
+  <si>
+    <t>thiyaguadmin</t>
   </si>
   <si>
     <t>Location</t>
   </si>
   <si>
+    <t>Hotels</t>
+  </si>
+  <si>
+    <t>Room Type</t>
+  </si>
+  <si>
     <t>Rooms</t>
   </si>
   <si>
-    <t>Arrival Date</t>
-  </si>
-  <si>
-    <t>Departure Date</t>
-  </si>
-  <si>
-    <t>No. of Days</t>
-  </si>
-  <si>
-    <t>Rooms Type</t>
-  </si>
-  <si>
-    <t>Price per Night</t>
-  </si>
-  <si>
-    <t>Total Price</t>
-  </si>
-  <si>
-    <t>1 Room</t>
-  </si>
-  <si>
-    <t>1 Day</t>
-  </si>
-  <si>
-    <t>AUD $ 125</t>
-  </si>
-  <si>
-    <t>AUD $ 135</t>
-  </si>
-  <si>
-    <t>2 Rooms</t>
-  </si>
-  <si>
-    <t>2 Days</t>
-  </si>
-  <si>
-    <t>AUD $ 275</t>
-  </si>
-  <si>
-    <t>AUD $ 285</t>
-  </si>
-  <si>
-    <t>Phone number</t>
-  </si>
-  <si>
-    <t>2 - Two</t>
-  </si>
-  <si>
-    <t>Hotels </t>
-  </si>
-  <si>
-    <t>Room Type</t>
-  </si>
-  <si>
-    <t>Number of Rooms</t>
-  </si>
-  <si>
     <t>Check In Date</t>
   </si>
   <si>
@@ -123,13 +81,46 @@
     <t>Children per Room</t>
   </si>
   <si>
-    <t>0 - None</t>
-  </si>
-  <si>
-    <t>3 - Three</t>
-  </si>
-  <si>
-    <t>1 - One</t>
+    <t>First Name</t>
+  </si>
+  <si>
+    <t>Last Name</t>
+  </si>
+  <si>
+    <t>Billing Address</t>
+  </si>
+  <si>
+    <t>Credit Card No</t>
+  </si>
+  <si>
+    <t>Credit Card Type</t>
+  </si>
+  <si>
+    <t>Expiry Month</t>
+  </si>
+  <si>
+    <t>Expiry Year</t>
+  </si>
+  <si>
+    <t>Deepak</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>5123 4567 8901 2346</t>
+  </si>
+  <si>
+    <t>February</t>
+  </si>
+  <si>
+    <t>No. 311, 122/B, Manickam Ave, Alwarpet, Chennai, Tamil Nadu 600018</t>
+  </si>
+  <si>
+    <t>CVV Number</t>
+  </si>
+  <si>
+    <t>Master Card</t>
   </si>
 </sst>
 </file>
@@ -173,11 +164,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -488,18 +478,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -512,7 +502,7 @@
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
@@ -523,43 +513,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>34</v>
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="E2" s="1">
         <v>46045</v>
@@ -568,24 +558,24 @@
         <v>46046</v>
       </c>
       <c r="G2" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="H2" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>27</v>
       </c>
       <c r="E3" s="1">
         <v>46045</v>
@@ -594,10 +584,10 @@
         <v>46045</v>
       </c>
       <c r="G3" t="s">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="H3" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -608,115 +598,69 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="1">
-        <v>46046</v>
-      </c>
-      <c r="E2" s="1">
-        <v>46047</v>
+        <v>32</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>34</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2">
-        <v>3423454345</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" s="1">
-        <v>46046</v>
-      </c>
-      <c r="E3" s="1">
-        <v>46047</v>
-      </c>
-      <c r="F3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3">
-        <v>2753498766</v>
+        <v>31</v>
+      </c>
+      <c r="G2">
+        <v>2027</v>
+      </c>
+      <c r="H2">
+        <v>533</v>
       </c>
     </row>
   </sheetData>

</xml_diff>